<commit_message>
Greek open-items document for Monada Elegchou Esodon
14 items needing a ruling, grouped by what each one blocks: two that stop the next
phase (the duplicate AET092 code and the 41 overlap pairs), four that stop costings
being finalised but not the build, and eight to close before go-live.

Generated by tools/make_questions_doc.py so every figure in it is read from the seed
data rather than typed. Re-runs after any seed change.

Also translates the overlap workbook headers to Greek, since the Monada is the one
filling it in.

No email sent.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LRcZ4u4yNRfNUeSzqtzBzE
</commit_message>
<xml_diff>
--- a/docs/overlap_decision_list.xlsx
+++ b/docs/overlap_decision_list.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Overlap decisions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Genuine extras" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Αποφάσεις επικάλυψης" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Πράγματι πρόσθετες" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Overlap decisions'!$A$1:$M$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Αποφάσεις επικάλυψης'!$A$1:$M$42</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -456,67 +456,67 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Service code</t>
+          <t>Κωδικός υπηρεσίας</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>Τύπος</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Cat</t>
+          <t>Κατ.</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Service description (EL)</t>
+          <t>Περιγραφή υπηρεσίας</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Tariff code</t>
+          <t>Κωδικός τιμοκαταλόγου</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Tariff description (EL)</t>
+          <t>Περιγραφή τιμοκαταλόγου</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Tariff price (raw)</t>
+          <t>Τιμή (όπως δόθηκε)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Tariff price €</t>
+          <t>Τιμή €</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Πρόταση</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>RULING (fill in)</t>
+          <t>ΑΠΟΦΑΣΗ (συμπληρώστε)</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Ruled by</t>
+          <t>Από</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Ruled on</t>
+          <t>Ημερομηνία</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Exposure €</t>
+          <t>Πρόσθετη χρέωση €</t>
         </is>
       </c>
     </row>
@@ -2565,7 +2565,7 @@
     <row r="44">
       <c r="I44" s="3" t="inlineStr">
         <is>
-          <t>Unruled pairs</t>
+          <t>Ζεύγη χωρίς απόφαση</t>
         </is>
       </c>
       <c r="J44" s="3">
@@ -2576,7 +2576,7 @@
     <row r="45">
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t>Exposure at current rulings €</t>
+          <t>Πρόσθετη χρέωση με τις τρέχουσες αποφάσεις €</t>
         </is>
       </c>
       <c r="J45" s="4">
@@ -2587,7 +2587,7 @@
     <row r="46">
       <c r="I46" s="3" t="inlineStr">
         <is>
-          <t>Exposure if all ruled 'both' €</t>
+          <t>Πρόσθετη χρέωση αν όλα κριθούν «both» €</t>
         </is>
       </c>
       <c r="J46" s="4">
@@ -2598,7 +2598,7 @@
   </sheetData>
   <autoFilter ref="A1:M42"/>
   <dataValidations count="1">
-    <dataValidation sqref="J2:J42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid ruling" error="Choose weight_only, tariff_only or both." type="list">
+    <dataValidation sqref="J2:J42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Μη έγκυρη απόφαση" error="Επιλέξτε weight_only, tariff_only ή both." type="list">
       <formula1>"weight_only,tariff_only,both"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2624,22 +2624,22 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Tariff code</t>
+          <t>Κωδικός</t>
         </is>
       </c>
       <c r="B1" s="5" t="inlineStr">
         <is>
-          <t>Description (EL)</t>
+          <t>Περιγραφή</t>
         </is>
       </c>
       <c r="C1" s="5" t="inlineStr">
         <is>
-          <t>Price (raw)</t>
+          <t>Τιμή (όπως δόθηκε)</t>
         </is>
       </c>
       <c r="D1" s="5" t="inlineStr">
         <is>
-          <t>Price €</t>
+          <t>Τιμή €</t>
         </is>
       </c>
     </row>

</xml_diff>